<commit_message>
docs: Update work diary
</commit_message>
<xml_diff>
--- a/Annexes/Journal_de_travail/Journal_de_Travail_DeCarvalho_Andre.xlsx
+++ b/Annexes/Journal_de_travail/Journal_de_Travail_DeCarvalho_Andre.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc38fqn\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ES\GITHUB\Lego-Inventor-Manager\Annexes\Journal_de_travail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686E2E3A-B6BF-4272-BE8F-FAA492C09481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B87A07C-D537-4753-B783-9CA3ECFD8A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="24">
   <si>
     <t>Jour</t>
   </si>
@@ -90,6 +90,27 @@
   </si>
   <si>
     <t>Configuration du depôt Git</t>
+  </si>
+  <si>
+    <t>Création du rapport de projet</t>
+  </si>
+  <si>
+    <t>Pris un peu de temps à réfléchir quoi poser comme information</t>
+  </si>
+  <si>
+    <t>Déterminer les tâches adaptées à leur niveau</t>
+  </si>
+  <si>
+    <t>Supervision du projet</t>
+  </si>
+  <si>
+    <t>Questions/Réponses</t>
+  </si>
+  <si>
+    <t>Réunion avec l'équipe et clarification des tâches</t>
+  </si>
+  <si>
+    <t>Solution apportée pour avoir un rythme linéaire</t>
   </si>
 </sst>
 </file>
@@ -805,7 +826,7 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -817,7 +838,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>1.3</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -826,7 +847,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1838,7 +1859,7 @@
   <dimension ref="A1:F500"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="26.625" style="4" customWidth="1"/>
     <col min="2" max="2" width="13.375" style="15" customWidth="1"/>
     <col min="3" max="3" width="15.25" style="12" customWidth="1"/>
     <col min="4" max="4" width="24.75" style="5" customWidth="1"/>
@@ -1903,36 +1924,82 @@
       <c r="F3" s="8"/>
     </row>
     <row r="4" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
+      <c r="A4" s="6">
+        <v>46036</v>
+      </c>
+      <c r="B4" s="14">
+        <v>1</v>
+      </c>
+      <c r="C4" s="11">
+        <v>1.3</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="8"/>
+      <c r="A5" s="6">
+        <v>46036</v>
+      </c>
+      <c r="B5" s="14">
+        <v>1</v>
+      </c>
+      <c r="C5" s="11">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="F5" s="8"/>
     </row>
     <row r="6" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
+      <c r="A6" s="6">
+        <v>46036</v>
+      </c>
+      <c r="B6" s="14">
+        <v>1</v>
+      </c>
+      <c r="C6" s="11">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
+      <c r="A7" s="6">
+        <v>46036</v>
+      </c>
+      <c r="B7" s="14">
+        <v>1</v>
+      </c>
+      <c r="C7" s="11">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
@@ -5935,7 +6002,7 @@
       </c>
       <c r="B2" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -5971,7 +6038,7 @@
       </c>
       <c r="B6" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>0</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -5998,7 +6065,7 @@
       </c>
       <c r="B9" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
docs: update working diary
</commit_message>
<xml_diff>
--- a/Annexes/Journal_de_travail/Journal_de_Travail_DeCarvalho_Andre.xlsx
+++ b/Annexes/Journal_de_travail/Journal_de_Travail_DeCarvalho_Andre.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ES\GITHUB\Lego-Inventor-Manager\Annexes\Journal_de_travail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22BC1F10-8274-468D-A11F-0659CCCD57A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44631F5D-99E6-4F65-8005-23A1011BF937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="40">
   <si>
     <t>Jour</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>Finalisation</t>
+  </si>
+  <si>
+    <t>Ajout des données mises à jour sur le MCD</t>
   </si>
 </sst>
 </file>
@@ -874,7 +877,7 @@
                   <c:v>2.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6</c:v>
+                  <c:v>6.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0.5</c:v>
@@ -2259,12 +2262,24 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="6"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
+      <c r="A19" s="6">
+        <v>46041</v>
+      </c>
+      <c r="B19" s="14">
+        <v>2</v>
+      </c>
+      <c r="C19" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
@@ -6204,7 +6219,7 @@
       </c>
       <c r="B3" s="11">
         <f>SUMIF(Journal!$D$2:$D$163,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$163)</f>
-        <v>6</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>